<commit_message>
materialeliste: tilføj sammenligning_beklaedning sheet
Sammenligner 6 reelle beklædnings-options ved 16 m² netto facadeareal:
imp. klinkbeklædning gran (billigst 2.593 kr), sortmalet klink 4200 (2.986),
Aros 1-på-2 (3.010), sortmalet lodret 3000 (4.672), høvlet fyr ubehandlet
(4.898), imp. høvlet fyr (5.176). Sorteret efter total pris, med Δ vs
billigste, farve-coded mønster-kolonne, klikbare leverandør-links.

Indeholder også behandlingsomkostning som separat kolonne så færdig-malede
produkter (klink sortmalet) sammenlignes fair mod råt træ der kræver
træolie/maling.
</commit_message>
<xml_diff>
--- a/docs/materialeliste.xlsx
+++ b/docs/materialeliste.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\privat\rabbit-house\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDC8518-F396-486B-96B5-99E425FFC517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7EB9800-5F23-42E0-85B4-522DC9A5F6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14070" yWindow="480" windowWidth="34095" windowHeight="18300" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6000" yWindow="690" windowWidth="34095" windowHeight="18300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
-    <sheet name="fundament" sheetId="2" r:id="rId2"/>
-    <sheet name="konstruktion" sheetId="3" r:id="rId3"/>
-    <sheet name="tagkonstruktion_tagpap" sheetId="4" r:id="rId4"/>
-    <sheet name="tagkonstruktion_eternit_b7" sheetId="5" r:id="rId5"/>
-    <sheet name="beklaedning_klink" sheetId="6" r:id="rId6"/>
-    <sheet name="beklaedning_board_on_board" sheetId="7" r:id="rId7"/>
+    <sheet name="sammenligning_beklaedning" sheetId="2" r:id="rId2"/>
+    <sheet name="fundament" sheetId="3" r:id="rId3"/>
+    <sheet name="konstruktion" sheetId="4" r:id="rId4"/>
+    <sheet name="tagkonstruktion_tagpap" sheetId="5" r:id="rId5"/>
+    <sheet name="tagkonstruktion_eternit_b7" sheetId="6" r:id="rId6"/>
+    <sheet name="beklaedning_klink" sheetId="7" r:id="rId7"/>
+    <sheet name="beklaedning_board_on_board" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="179">
   <si>
     <t>Rabbit-house BOM  —  variant selector</t>
   </si>
@@ -95,27 +96,171 @@
     <t>Noter</t>
   </si>
   <si>
+    <t>•  Dropdowns i B3/B4 styrer totalen i B11 via INDIRECT på sheet-navne.</t>
+  </si>
+  <si>
+    <t>•  Eternit_b7 bruger tungere spær (47×100 C24) end tagpap (men prisen er fra eternit-doc og er et estimat).</t>
+  </si>
+  <si>
+    <t>•  Board-on-board pris er Aros tilbudspris 160 kr/m² (normalpris 225). Klink kommer sortmalet; bob behøver træolie/maling.</t>
+  </si>
+  <si>
+    <t>•  Voliernet og isolering er ens på tværs af beklædningsvarianter.</t>
+  </si>
+  <si>
+    <t>•  Variantvalg i build.scad: roof_cover = "tagpap_osb"|"eternit_b7"; cladding_type = "klink"|"board_on_board".</t>
+  </si>
+  <si>
+    <t>•  Items med pris=tom og noter="TBD …" kræver verifikation før bestilling.</t>
+  </si>
+  <si>
+    <t>Beklædning — prissammenligning ved 16 m² netto facadeareal</t>
+  </si>
+  <si>
+    <t>Produkt</t>
+  </si>
+  <si>
+    <t>Mønster</t>
+  </si>
+  <si>
+    <t>Materiale</t>
+  </si>
+  <si>
+    <t>Antal</t>
+  </si>
+  <si>
+    <t>Enhed</t>
+  </si>
+  <si>
+    <t>Pris/enh</t>
+  </si>
+  <si>
+    <t>Material kr</t>
+  </si>
+  <si>
+    <t>Behandl. kr</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Δ vs billigst</t>
+  </si>
+  <si>
+    <t>Leverandør</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Imp. klinkbeklædning gran 25×125×3600</t>
+  </si>
+  <si>
+    <t>Klink horisontal</t>
+  </si>
+  <si>
+    <t>Trykimp. gran (ubehandlet ud over imp.)</t>
+  </si>
+  <si>
+    <t>stk</t>
+  </si>
+  <si>
+    <t>jemogfix.dk</t>
+  </si>
+  <si>
+    <t>Billigste klink. Grøn-grålig fra start; kan males sort senere (+~450 kr)</t>
+  </si>
+  <si>
+    <t>Klinkbeklædning sortmalet gran 25×125×4200 (6-pak)</t>
+  </si>
+  <si>
+    <t>Gran, færdig sortmalet vandbaseret RAL 9005</t>
+  </si>
+  <si>
+    <t>pak</t>
+  </si>
+  <si>
+    <t>Klar til at montere. Klassisk skur/sommerhus-look. 6 stk pr. pak = 25,2 m linear</t>
+  </si>
+  <si>
+    <t>Aros 1-på-2 svensk gran 25×150 savskåret</t>
+  </si>
+  <si>
+    <t>1-på-2 lodret (bob)</t>
+  </si>
+  <si>
+    <t>Savskåret svensk gran (FSC)</t>
+  </si>
+  <si>
+    <t>m²</t>
+  </si>
+  <si>
+    <t>arossavvaerk.dk</t>
+  </si>
+  <si>
+    <t>Tilbudspris 160 (normal 225). Rustic look. Behandling påkrævet før montage</t>
+  </si>
+  <si>
+    <t>Beklædning lodret sort 25×125×3000 (4-pak)</t>
+  </si>
+  <si>
+    <t>Klink lodret</t>
+  </si>
+  <si>
+    <t>Skandinavisk gran (FSC), færdig sortmalet vandbaseret</t>
+  </si>
+  <si>
+    <t>Lodret klink-profil, færdig sort. 4 stk pr. pak = 12 m linear. Moderne lade-look</t>
+  </si>
+  <si>
+    <t>Høvlet forskalling fyr 22×100×3600 UBEHANDLET</t>
+  </si>
+  <si>
+    <t>Fyr, høvlet, ubehandlet</t>
+  </si>
+  <si>
+    <t>Jemogfix advarer mod udendørs ubehandlet. Kræver Gori/Pinotex × 3 lag</t>
+  </si>
+  <si>
+    <t>Imprægneret høvlet fyr 25×125×3600</t>
+  </si>
+  <si>
+    <t>Trykimp. fyr, høvlet</t>
+  </si>
+  <si>
+    <t>Udendørs-godkendt. Grøn-brun farve fra imp. Kan males (+~450 kr)</t>
+  </si>
+  <si>
+    <t>Læsevejledning</t>
+  </si>
+  <si>
+    <t>•  Antal er beregnet for 16 m² netto vægareal (4 hus-vægge minus side-vindue + dør + kanindør).</t>
+  </si>
+  <si>
+    <t>•  Behandl. kr = ekstra behandlingsomkostning (træolie/maling) der KRÆVES før montage. 0 hvis produktet er færdigbehandlet eller trykimp.</t>
+  </si>
+  <si>
+    <t>•  Klink-produkter har færdig profil (overlapper indbygget). 1-på-2 (bob) bruger to lag rå brædder; kræver mere arbejde at montere.</t>
+  </si>
+  <si>
+    <t>•  Mønster-farven matcher beklædnings-sheet i resten af workbook'en: blå = klink, grøn = bob, gul = lodret klink.</t>
+  </si>
+  <si>
+    <t>•  TOTAL inkluderer IKKE: voliernet, vindpap, klemmelister, isolering, hjørnetrim (~2.000-2.500 kr fælles, se beklaedning_* sheets).</t>
+  </si>
+  <si>
     <t>Kategori</t>
   </si>
   <si>
     <t>Vare</t>
   </si>
   <si>
-    <t>Antal</t>
-  </si>
-  <si>
-    <t>Enhed</t>
-  </si>
-  <si>
     <t>Pris pr. enhed (DKK)</t>
   </si>
   <si>
     <t>I alt (DKK)</t>
   </si>
   <si>
-    <t>Leverandør</t>
-  </si>
-  <si>
     <t>Stabilgrus 0-32 mm</t>
   </si>
   <si>
@@ -131,12 +276,6 @@
     <t>Fundablok 50x20x15 cm</t>
   </si>
   <si>
-    <t>stk</t>
-  </si>
-  <si>
-    <t>jemogfix.dk</t>
-  </si>
-  <si>
     <t>Behov 117 stk; købes 120</t>
   </si>
   <si>
@@ -173,9 +312,6 @@
     <t>NKT Fasteners</t>
   </si>
   <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
     <t>Murpap (DPC)</t>
   </si>
   <si>
@@ -281,9 +417,6 @@
     <t>Paslode vinkelbeslag 90×90×40 (20-pak)</t>
   </si>
   <si>
-    <t>pak</t>
-  </si>
-  <si>
     <t>wood-online.dk</t>
   </si>
   <si>
@@ -308,15 +441,27 @@
     <t>Alusøm</t>
   </si>
   <si>
+    <t>Stark</t>
+  </si>
+  <si>
     <t>est. — Stark; tungere end tagpap</t>
   </si>
   <si>
     <t>C18 taglægte 38×73×4200 mm</t>
   </si>
   <si>
+    <t>10-4.dk</t>
+  </si>
+  <si>
     <t>6 rækker à ~6,44 m + spild</t>
   </si>
   <si>
+    <t>Imp. sternbræt 25×125×3600 gran</t>
+  </si>
+  <si>
+    <t>xl-byg.dk</t>
+  </si>
+  <si>
     <t>Hele perimeter ~19 m</t>
   </si>
   <si>
@@ -395,16 +540,10 @@
     <t>Isolering mineraluld 95 mm</t>
   </si>
   <si>
-    <t>m²</t>
-  </si>
-  <si>
     <t>I stud-rum, 2 vægge ~6 m² + 2 vægge ~4 m²</t>
   </si>
   <si>
     <t>1-på-2 svensk gran 25×150 savskåret</t>
-  </si>
-  <si>
-    <t>arossavvaerk.dk</t>
   </si>
   <si>
     <t>Aros tilbudspris; normal 225 kr/m²</t>
@@ -444,8 +583,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;kr&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0\ &quot;kr&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -493,12 +633,10 @@
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="14">
@@ -593,11 +731,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -642,15 +779,37 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -674,18 +833,20 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1018,7 +1179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -1027,12 +1188,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.95" customHeight="1">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
@@ -1051,12 +1212,12 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="20.100000000000001" customHeight="1">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="5" t="s">
@@ -1091,7 +1252,7 @@
       </c>
       <c r="B10" s="6">
         <f ca="1">SUM(INDIRECT("beklaedning_"&amp;B4&amp;"!F:F"))</f>
-        <v>5035.7</v>
+        <v>6977.9</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75">
@@ -1100,16 +1261,16 @@
       </c>
       <c r="B11" s="10">
         <f ca="1">SUM(B7:B10)</f>
-        <v>21716.000000000004</v>
+        <v>23658.200000000004</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="20.100000000000001" customHeight="1">
-      <c r="A13" s="46" t="s">
+      <c r="A13" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
     </row>
     <row r="14" spans="1:4">
       <c r="B14" s="11" t="s">
@@ -1128,15 +1289,15 @@
       </c>
       <c r="B15" s="6">
         <f>SUM(fundament!F:F)+SUM(konstruktion!F:F)+SUM(tagkonstruktion_tagpap!F:F)+SUM(beklaedning_klink!F:F)</f>
-        <v>21716.000000000004</v>
+        <v>23658.200000000004</v>
       </c>
       <c r="C15" s="6">
         <f>SUM(fundament!F:F)+SUM(konstruktion!F:F)+SUM(tagkonstruktion_eternit_b7!F:F)+SUM(beklaedning_klink!F:F)</f>
-        <v>21801.750000000004</v>
+        <v>24038.35</v>
       </c>
       <c r="D15" s="15">
         <f>C15-B15</f>
-        <v>85.75</v>
+        <v>380.14999999999418</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1145,15 +1306,15 @@
       </c>
       <c r="B16" s="6">
         <f>SUM(fundament!F:F)+SUM(konstruktion!F:F)+SUM(tagkonstruktion_tagpap!F:F)+SUM(beklaedning_board_on_board!F:F)</f>
-        <v>21172.800000000003</v>
+        <v>23115.000000000004</v>
       </c>
       <c r="C16" s="6">
         <f>SUM(fundament!F:F)+SUM(konstruktion!F:F)+SUM(tagkonstruktion_eternit_b7!F:F)+SUM(beklaedning_board_on_board!F:F)</f>
-        <v>21258.550000000003</v>
+        <v>23495.15</v>
       </c>
       <c r="D16" s="15">
         <f>C16-B16</f>
-        <v>85.75</v>
+        <v>380.14999999999782</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1166,50 +1327,78 @@
       </c>
       <c r="C17" s="15">
         <f>C16-C15</f>
-        <v>-543.20000000000073</v>
+        <v>-543.19999999999709</v>
       </c>
       <c r="D17" s="18"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="44"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
+      <c r="A19" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="55"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="44"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
+      <c r="A20" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="44"/>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
+      <c r="A21" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="44"/>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
+      <c r="A22" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="55"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="44"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
+      <c r="A23" s="56" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="55"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="55"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A22:D22"/>
+  <mergeCells count="10">
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" sqref="B3" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1225,6 +1414,440 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="24" customHeight="1">
+      <c r="A1" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1">
+      <c r="A3" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="22">
+        <v>43</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="24">
+        <v>60.3</v>
+      </c>
+      <c r="G4" s="25">
+        <f t="shared" ref="G4:G9" si="0">D4*F4</f>
+        <v>2592.9</v>
+      </c>
+      <c r="H4" s="26">
+        <v>0</v>
+      </c>
+      <c r="I4" s="27">
+        <f t="shared" ref="I4:I9" si="1">G4+H4</f>
+        <v>2592.9</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="K4" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="22">
+        <v>6</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="24">
+        <v>497.7</v>
+      </c>
+      <c r="G5" s="25">
+        <f t="shared" si="0"/>
+        <v>2986.2</v>
+      </c>
+      <c r="H5" s="26">
+        <v>0</v>
+      </c>
+      <c r="I5" s="30">
+        <f t="shared" si="1"/>
+        <v>2986.2</v>
+      </c>
+      <c r="J5" s="15">
+        <v>393.29999999999973</v>
+      </c>
+      <c r="K5" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" s="29" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="22">
+        <v>16</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="24">
+        <v>160</v>
+      </c>
+      <c r="G6" s="25">
+        <f t="shared" si="0"/>
+        <v>2560</v>
+      </c>
+      <c r="H6" s="26">
+        <v>450</v>
+      </c>
+      <c r="I6" s="30">
+        <f t="shared" si="1"/>
+        <v>3010</v>
+      </c>
+      <c r="J6" s="15">
+        <v>417.09999999999991</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" s="29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="22">
+        <v>13</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="24">
+        <v>359.4</v>
+      </c>
+      <c r="G7" s="25">
+        <f t="shared" si="0"/>
+        <v>4672.2</v>
+      </c>
+      <c r="H7" s="26">
+        <v>0</v>
+      </c>
+      <c r="I7" s="30">
+        <f t="shared" si="1"/>
+        <v>4672.2</v>
+      </c>
+      <c r="J7" s="15">
+        <v>2079.3000000000002</v>
+      </c>
+      <c r="K7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="L7" s="29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="22">
+        <v>120</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="24">
+        <v>35.82</v>
+      </c>
+      <c r="G8" s="25">
+        <f t="shared" si="0"/>
+        <v>4298.3999999999996</v>
+      </c>
+      <c r="H8" s="26">
+        <v>600</v>
+      </c>
+      <c r="I8" s="30">
+        <f t="shared" si="1"/>
+        <v>4898.3999999999996</v>
+      </c>
+      <c r="J8" s="15">
+        <v>2305.5</v>
+      </c>
+      <c r="K8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" s="29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="22">
+        <v>81</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="24">
+        <v>63.9</v>
+      </c>
+      <c r="G9" s="25">
+        <f t="shared" si="0"/>
+        <v>5175.8999999999996</v>
+      </c>
+      <c r="H9" s="26">
+        <v>0</v>
+      </c>
+      <c r="I9" s="30">
+        <f t="shared" si="1"/>
+        <v>5175.8999999999996</v>
+      </c>
+      <c r="J9" s="15">
+        <v>2583</v>
+      </c>
+      <c r="K9" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="56" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="55"/>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" s="56" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="55"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="55"/>
+      <c r="L15" s="55"/>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" s="56" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="55"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="56" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="55"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="55"/>
+      <c r="I17" s="55"/>
+      <c r="J17" s="55"/>
+      <c r="K17" s="55"/>
+      <c r="L17" s="55"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A12:F12"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="K5" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="K6" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="K7" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="K8" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="K9" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1238,28 +1861,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1268,188 +1891,188 @@
         <v>6</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C2" s="18">
         <v>1050</v>
       </c>
-      <c r="D2" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="21">
+      <c r="D2" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="24">
         <v>0.55000000000000004</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="24">
         <f t="shared" ref="F2:F8" si="0">C2*E2</f>
         <v>577.5</v>
       </c>
-      <c r="G2" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>28</v>
+      <c r="G2" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="C3" s="18">
         <v>120</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21">
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24">
         <v>15.75</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="24">
         <f t="shared" si="0"/>
         <v>1890</v>
       </c>
-      <c r="G3" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>32</v>
+      <c r="G3" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="C4" s="18">
         <v>13</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="21">
+      <c r="D4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="24">
         <v>29.75</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="24">
         <f t="shared" si="0"/>
         <v>386.75</v>
       </c>
-      <c r="G4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>34</v>
+      <c r="G4" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="C5" s="18">
         <v>14</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="D5" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="24">
         <v>75</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="24">
         <f t="shared" si="0"/>
         <v>1050</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="23" t="s">
-        <v>36</v>
+      <c r="G5" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="C6" s="18">
         <v>1485</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="21">
+      <c r="D6" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="24">
         <v>0.66</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="24">
         <f t="shared" si="0"/>
         <v>980.1</v>
       </c>
-      <c r="G6" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>38</v>
+      <c r="G6" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>39</v>
+        <v>85</v>
       </c>
       <c r="C7" s="18">
         <v>18</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="21">
+      <c r="D7" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="24">
         <v>27.95</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="24">
         <f t="shared" si="0"/>
         <v>503.09999999999997</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>40</v>
+      <c r="G7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
       <c r="C8" s="18">
         <v>2</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="D8" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="24">
         <v>28.95</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="24">
         <f t="shared" si="0"/>
         <v>57.9</v>
       </c>
-      <c r="G8" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>43</v>
+      <c r="G8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1457,220 +2080,18 @@
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="25"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="18"/>
       <c r="C10" s="18"/>
       <c r="D10" s="18"/>
-      <c r="E10" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="21"/>
+      <c r="E10" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="24"/>
       <c r="G10" s="18"/>
-      <c r="H10" s="27">
+      <c r="H10" s="37">
         <f>SUM(F2:F8)</f>
         <v>5445.35</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="G7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="G8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="60" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="18">
-        <v>1</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="21">
-        <v>99</v>
-      </c>
-      <c r="F2" s="21">
-        <f>C2*E2</f>
-        <v>99</v>
-      </c>
-      <c r="G2" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="18">
-        <v>2</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21">
-        <v>71.099999999999994</v>
-      </c>
-      <c r="F3" s="21">
-        <f>C3*E3</f>
-        <v>142.19999999999999</v>
-      </c>
-      <c r="G3" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="18">
-        <v>5</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="21">
-        <v>47.4</v>
-      </c>
-      <c r="F4" s="21">
-        <f>C4*E4</f>
-        <v>237</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="23"/>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" s="18">
-        <v>4</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="21">
-        <v>63.9</v>
-      </c>
-      <c r="F5" s="21">
-        <f>C5*E5</f>
-        <v>255.6</v>
-      </c>
-      <c r="G5" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="23"/>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="18">
-        <v>42</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="21">
-        <v>42.6</v>
-      </c>
-      <c r="F6" s="21">
-        <f>C6*E6</f>
-        <v>1789.2</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="29"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="27">
-        <f>SUM(F2:F6)</f>
-        <v>2523</v>
       </c>
     </row>
   </sheetData>
@@ -1680,6 +2101,8 @@
     <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
     <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
     <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1687,6 +2110,206 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="21.95" customHeight="1">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="18">
+        <v>1</v>
+      </c>
+      <c r="D2" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="24">
+        <v>99</v>
+      </c>
+      <c r="F2" s="24">
+        <f>C2*E2</f>
+        <v>99</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="18">
+        <v>2</v>
+      </c>
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="F3" s="24">
+        <f>C3*E3</f>
+        <v>142.19999999999999</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="29"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="18">
+        <v>5</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="24">
+        <v>47.4</v>
+      </c>
+      <c r="F4" s="24">
+        <f>C4*E4</f>
+        <v>237</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="29"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="18">
+        <v>4</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="24">
+        <v>63.9</v>
+      </c>
+      <c r="F5" s="24">
+        <f>C5*E5</f>
+        <v>255.6</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="29"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="18">
+        <v>42</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="24">
+        <v>42.6</v>
+      </c>
+      <c r="F6" s="24">
+        <f>C6*E6</f>
+        <v>1789.2</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="39"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="24"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="37">
+        <f>SUM(F2:F6)</f>
+        <v>2523</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1700,108 +2323,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="30" t="s">
-        <v>52</v>
+      <c r="A2" s="40" t="s">
+        <v>97</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="C2" s="18">
         <v>13</v>
       </c>
-      <c r="D2" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="21">
+      <c r="D2" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="24">
         <v>53.25</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="24">
         <f>C2*E2</f>
         <v>692.25</v>
       </c>
-      <c r="G2" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" s="23"/>
+      <c r="G2" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="31" t="s">
-        <v>52</v>
+      <c r="A3" s="41" t="s">
+        <v>97</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="C3" s="18">
         <v>15</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21">
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24">
         <v>129</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="24">
         <f>C3*E3</f>
         <v>1935</v>
       </c>
-      <c r="G3" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>55</v>
+      <c r="G3" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="31" t="s">
-        <v>52</v>
+      <c r="A4" s="41" t="s">
+        <v>97</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C4" s="18">
         <v>6</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="21">
+      <c r="D4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="24">
         <v>92.7</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="24">
         <f>C4*E4</f>
         <v>556.20000000000005</v>
       </c>
-      <c r="G4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>57</v>
+      <c r="G4" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1809,342 +2432,342 @@
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="30" t="s">
-        <v>58</v>
+      <c r="A6" s="40" t="s">
+        <v>103</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="C6" s="18">
         <v>5</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="21">
+      <c r="D6" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="24">
         <v>579</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="24">
         <f>C6*E6</f>
         <v>2895</v>
       </c>
-      <c r="G6" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="23"/>
+      <c r="G6" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="29"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="31" t="s">
-        <v>58</v>
+      <c r="A7" s="41" t="s">
+        <v>103</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="C7" s="18">
         <v>3</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="21">
+      <c r="D7" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="24">
         <v>69.95</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="24">
         <f>C7*E7</f>
         <v>209.85000000000002</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="23"/>
+      <c r="G7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="29"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="31" t="s">
-        <v>58</v>
+      <c r="A8" s="41" t="s">
+        <v>103</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>61</v>
+        <v>106</v>
       </c>
       <c r="C8" s="18">
         <v>1</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="D8" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="24">
         <v>149</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="24">
         <f>C8*E8</f>
         <v>149</v>
       </c>
-      <c r="G8" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="23"/>
+      <c r="G8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="29"/>
     </row>
     <row r="9" spans="1:8">
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="30" t="s">
-        <v>62</v>
+      <c r="A10" s="40" t="s">
+        <v>107</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="C10" s="18">
         <v>7</v>
       </c>
-      <c r="D10" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="21">
+      <c r="D10" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="24">
         <v>39.75</v>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="24">
         <f>C10*E10</f>
         <v>278.25</v>
       </c>
-      <c r="G10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="23"/>
+      <c r="G10" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="29"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="31" t="s">
-        <v>62</v>
+      <c r="A11" s="41" t="s">
+        <v>107</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="C11" s="18">
         <v>13</v>
       </c>
-      <c r="D11" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="21">
+      <c r="D11" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="24">
         <v>59.95</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="24">
         <f>C11*E11</f>
         <v>779.35</v>
       </c>
-      <c r="G11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="23"/>
+      <c r="G11" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" spans="1:8">
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="30" t="s">
-        <v>65</v>
+      <c r="A13" s="40" t="s">
+        <v>110</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="C13" s="18">
         <v>7</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="E13" s="21">
+      <c r="D13" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="E13" s="24">
         <v>49.95</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="24">
         <f t="shared" ref="F13:F20" si="0">C13*E13</f>
         <v>349.65000000000003</v>
       </c>
-      <c r="G13" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13" s="23"/>
+      <c r="G13" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="31" t="s">
-        <v>65</v>
+      <c r="A14" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="C14" s="18">
         <v>10</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" s="21">
+      <c r="D14" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="24">
         <v>24.95</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="24">
         <f t="shared" si="0"/>
         <v>249.5</v>
       </c>
-      <c r="G14" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>69</v>
+      <c r="G14" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="29" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="31" t="s">
-        <v>65</v>
+      <c r="A15" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="C15" s="18">
         <v>1</v>
       </c>
-      <c r="D15" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="21">
+      <c r="D15" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="24">
         <v>46.75</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="24">
         <f t="shared" si="0"/>
         <v>46.75</v>
       </c>
-      <c r="G15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H15" s="23"/>
+      <c r="G15" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="31" t="s">
-        <v>65</v>
+      <c r="A16" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>71</v>
+        <v>116</v>
       </c>
       <c r="C16" s="18">
         <v>2</v>
       </c>
-      <c r="D16" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" s="21">
+      <c r="D16" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="24">
         <v>43.75</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="24">
         <f t="shared" si="0"/>
         <v>87.5</v>
       </c>
-      <c r="G16" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H16" s="23"/>
+      <c r="G16" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="31" t="s">
-        <v>65</v>
+      <c r="A17" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="C17" s="18">
         <v>1</v>
       </c>
-      <c r="D17" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" s="21">
+      <c r="D17" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="24">
         <v>19.95</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="24">
         <f t="shared" si="0"/>
         <v>19.95</v>
       </c>
-      <c r="G17" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H17" s="23"/>
+      <c r="G17" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="31" t="s">
-        <v>65</v>
+      <c r="A18" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="C18" s="18">
         <v>1</v>
       </c>
-      <c r="D18" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="21">
+      <c r="D18" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="24">
         <v>210</v>
       </c>
-      <c r="F18" s="21">
+      <c r="F18" s="24">
         <f t="shared" si="0"/>
         <v>210</v>
       </c>
-      <c r="G18" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>74</v>
+      <c r="G18" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="29" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="31" t="s">
-        <v>65</v>
+      <c r="A19" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="C19" s="18">
         <v>1</v>
       </c>
-      <c r="D19" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" s="21">
+      <c r="D19" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="24">
         <v>78.75</v>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="24">
         <f t="shared" si="0"/>
         <v>78.75</v>
       </c>
-      <c r="G19" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="23"/>
+      <c r="G19" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="31" t="s">
-        <v>65</v>
+      <c r="A20" s="41" t="s">
+        <v>110</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="C20" s="18">
         <v>1</v>
       </c>
-      <c r="D20" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20" s="21">
+      <c r="D20" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="24">
         <v>105</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="24">
         <f t="shared" si="0"/>
         <v>105</v>
       </c>
-      <c r="G20" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H20" s="23" t="s">
-        <v>77</v>
+      <c r="G20" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" s="29" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2152,94 +2775,94 @@
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="30" t="s">
-        <v>78</v>
+      <c r="A22" s="40" t="s">
+        <v>123</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="C22" s="18">
         <v>3</v>
       </c>
-      <c r="D22" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="H22" s="23" t="s">
-        <v>82</v>
+      <c r="D22" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="H22" s="29" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="31" t="s">
-        <v>78</v>
+      <c r="A23" s="41" t="s">
+        <v>123</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="C23" s="18">
         <v>250</v>
       </c>
-      <c r="D23" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
+      <c r="D23" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
       <c r="G23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H23" s="23" t="s">
-        <v>84</v>
+        <v>41</v>
+      </c>
+      <c r="H23" s="29" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="31" t="s">
-        <v>78</v>
+      <c r="A24" s="41" t="s">
+        <v>123</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>85</v>
+        <v>129</v>
       </c>
       <c r="C24" s="18"/>
-      <c r="D24" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="D24" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
       <c r="G24" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H24" s="23" t="s">
-        <v>86</v>
+        <v>41</v>
+      </c>
+      <c r="H24" s="29" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="31" t="s">
-        <v>78</v>
+      <c r="A25" s="41" t="s">
+        <v>123</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>87</v>
+        <v>131</v>
       </c>
       <c r="C25" s="18">
         <v>1</v>
       </c>
-      <c r="D25" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="21">
+      <c r="D25" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="24">
         <v>69.95</v>
       </c>
-      <c r="F25" s="21">
+      <c r="F25" s="24">
         <f>C25*E25</f>
         <v>69.95</v>
       </c>
-      <c r="G25" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H25" s="23" t="s">
-        <v>88</v>
+      <c r="G25" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H25" s="29" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2247,47 +2870,47 @@
       <c r="F26" s="1"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="32"/>
+      <c r="A27" s="42"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
       <c r="D27" s="18"/>
-      <c r="E27" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F27" s="21"/>
+      <c r="E27" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="24"/>
       <c r="G27" s="18"/>
-      <c r="H27" s="27">
+      <c r="H27" s="37">
         <f>SUM(F2:F25)</f>
         <v>8711.9500000000007</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="G6" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
-    <hyperlink ref="G7" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
-    <hyperlink ref="G8" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
-    <hyperlink ref="G10" r:id="rId7" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
-    <hyperlink ref="G11" r:id="rId8" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
-    <hyperlink ref="G13" r:id="rId9" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
-    <hyperlink ref="G14" r:id="rId10" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
-    <hyperlink ref="G15" r:id="rId11" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
-    <hyperlink ref="G16" r:id="rId12" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
-    <hyperlink ref="G17" r:id="rId13" xr:uid="{00000000-0004-0000-0300-00000C000000}"/>
-    <hyperlink ref="G18" r:id="rId14" xr:uid="{00000000-0004-0000-0300-00000D000000}"/>
-    <hyperlink ref="G19" r:id="rId15" xr:uid="{00000000-0004-0000-0300-00000E000000}"/>
-    <hyperlink ref="G20" r:id="rId16" xr:uid="{00000000-0004-0000-0300-00000F000000}"/>
-    <hyperlink ref="G22" r:id="rId17" xr:uid="{00000000-0004-0000-0300-000010000000}"/>
-    <hyperlink ref="G25" r:id="rId18" xr:uid="{00000000-0004-0000-0300-000011000000}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="G7" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="G8" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="G10" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="G11" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="G13" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="G14" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="G15" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="G16" r:id="rId12" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="G17" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="G18" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="G19" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="G20" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="G22" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="G25" r:id="rId18" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2301,110 +2924,110 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="33" t="s">
-        <v>52</v>
+      <c r="A2" s="43" t="s">
+        <v>97</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="C2" s="18">
         <v>13</v>
       </c>
-      <c r="D2" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="21">
-        <v>53.25</v>
-      </c>
-      <c r="F2" s="21">
+      <c r="D2" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="24">
+        <v>85</v>
+      </c>
+      <c r="F2" s="24">
         <f>C2*E2</f>
-        <v>692.25</v>
-      </c>
-      <c r="G2" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>89</v>
+        <v>1105</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="34" t="s">
-        <v>52</v>
+      <c r="A3" s="44" t="s">
+        <v>97</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="C3" s="18">
         <v>11</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21">
-        <v>57.75</v>
-      </c>
-      <c r="F3" s="21">
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24">
+        <v>52.5</v>
+      </c>
+      <c r="F3" s="24">
         <f>C3*E3</f>
-        <v>635.25</v>
-      </c>
-      <c r="G3" s="48" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>91</v>
+        <v>577.5</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="34" t="s">
-        <v>52</v>
+      <c r="A4" s="44" t="s">
+        <v>97</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>56</v>
+        <v>138</v>
       </c>
       <c r="C4" s="18">
         <v>6</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="21">
-        <v>92.7</v>
-      </c>
-      <c r="F4" s="21">
+      <c r="D4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="24">
+        <v>82.6</v>
+      </c>
+      <c r="F4" s="24">
         <f>C4*E4</f>
-        <v>556.20000000000005</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>92</v>
+        <v>495.59999999999997</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>139</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2412,79 +3035,79 @@
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="33" t="s">
-        <v>58</v>
+      <c r="A6" s="43" t="s">
+        <v>103</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="C6" s="18">
         <v>52</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="21">
+      <c r="D6" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="24">
         <v>95</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="24">
         <f>C6*E6</f>
         <v>4940</v>
       </c>
-      <c r="G6" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>95</v>
+      <c r="G6" s="28" t="s">
+        <v>142</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="34" t="s">
-        <v>58</v>
+      <c r="A7" s="44" t="s">
+        <v>103</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="C7" s="18">
         <v>2</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="21">
+      <c r="D7" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="24">
         <v>425</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="24">
         <f>C7*E7</f>
         <v>850</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>98</v>
+      <c r="G7" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="34" t="s">
-        <v>58</v>
+      <c r="A8" s="44" t="s">
+        <v>103</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="C8" s="18">
         <v>1</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
+      <c r="D8" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
       <c r="G8" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>102</v>
+        <v>149</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2492,201 +3115,201 @@
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="33" t="s">
-        <v>65</v>
+      <c r="A10" s="43" t="s">
+        <v>110</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="C10" s="18">
         <v>7</v>
       </c>
-      <c r="D10" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" s="21">
+      <c r="D10" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" s="24">
         <v>49.95</v>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="24">
         <f t="shared" ref="F10:F15" si="0">C10*E10</f>
         <v>349.65000000000003</v>
       </c>
-      <c r="G10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="23"/>
+      <c r="G10" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="29"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="34" t="s">
-        <v>65</v>
+      <c r="A11" s="44" t="s">
+        <v>110</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="C11" s="18">
         <v>12</v>
       </c>
-      <c r="D11" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="21">
+      <c r="D11" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="24">
         <v>24.95</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="24">
         <f t="shared" si="0"/>
         <v>299.39999999999998</v>
       </c>
-      <c r="G11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="23" t="s">
-        <v>69</v>
+      <c r="G11" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H11" s="29" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="34" t="s">
-        <v>65</v>
+      <c r="A12" s="44" t="s">
+        <v>110</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>71</v>
+        <v>116</v>
       </c>
       <c r="C12" s="18">
         <v>2</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="21">
+      <c r="D12" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="24">
         <v>43.75</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="24">
         <f t="shared" si="0"/>
         <v>87.5</v>
       </c>
-      <c r="G12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="23"/>
+      <c r="G12" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="34" t="s">
-        <v>65</v>
+      <c r="A13" s="44" t="s">
+        <v>110</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="C13" s="18">
         <v>1</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="21">
+      <c r="D13" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="24">
         <v>19.95</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="24">
         <f t="shared" si="0"/>
         <v>19.95</v>
       </c>
-      <c r="G13" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13" s="23"/>
+      <c r="G13" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="34" t="s">
-        <v>65</v>
+      <c r="A14" s="44" t="s">
+        <v>110</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="C14" s="18">
         <v>1</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" s="21">
+      <c r="D14" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="24">
         <v>210</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="24">
         <f t="shared" si="0"/>
         <v>210</v>
       </c>
-      <c r="G14" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" s="23"/>
+      <c r="G14" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="34" t="s">
-        <v>65</v>
+      <c r="A15" s="44" t="s">
+        <v>110</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="C15" s="18">
         <v>2</v>
       </c>
-      <c r="D15" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="21">
+      <c r="D15" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="24">
         <v>78.75</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="24">
         <f t="shared" si="0"/>
         <v>157.5</v>
       </c>
-      <c r="G15" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H15" s="23"/>
+      <c r="G15" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="1:8">
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="33" t="s">
-        <v>78</v>
+      <c r="A17" s="43" t="s">
+        <v>123</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="C17" s="18">
         <v>3</v>
       </c>
-      <c r="D17" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="H17" s="23" t="s">
-        <v>82</v>
+      <c r="D17" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="H17" s="29" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="34" t="s">
-        <v>78</v>
+      <c r="A18" s="44" t="s">
+        <v>123</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>103</v>
+        <v>151</v>
       </c>
       <c r="C18" s="18"/>
-      <c r="D18" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
+      <c r="D18" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
       <c r="G18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>86</v>
+        <v>41</v>
+      </c>
+      <c r="H18" s="29" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -2694,41 +3317,41 @@
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="35"/>
+      <c r="A20" s="45"/>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
-      <c r="E20" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F20" s="21"/>
+      <c r="E20" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="24"/>
       <c r="G20" s="18"/>
-      <c r="H20" s="27">
+      <c r="H20" s="37">
         <f>SUM(F2:F18)</f>
-        <v>8797.7000000000007</v>
+        <v>9092.1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
-    <hyperlink ref="G10" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
-    <hyperlink ref="G11" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
-    <hyperlink ref="G12" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
-    <hyperlink ref="G13" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
-    <hyperlink ref="G14" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
-    <hyperlink ref="G15" r:id="rId9" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
-    <hyperlink ref="G17" r:id="rId10" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
-    <hyperlink ref="G2" r:id="rId11" xr:uid="{1F4150C7-3DA7-4523-897D-511C468BC6AB}"/>
-    <hyperlink ref="G4" r:id="rId12" xr:uid="{0E4E6C89-09C1-4E2D-8483-CB6834E6D365}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
+    <hyperlink ref="G7" r:id="rId5" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
+    <hyperlink ref="G10" r:id="rId6" xr:uid="{00000000-0004-0000-0500-000005000000}"/>
+    <hyperlink ref="G11" r:id="rId7" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
+    <hyperlink ref="G12" r:id="rId8" xr:uid="{00000000-0004-0000-0500-000007000000}"/>
+    <hyperlink ref="G13" r:id="rId9" xr:uid="{00000000-0004-0000-0500-000008000000}"/>
+    <hyperlink ref="G14" r:id="rId10" xr:uid="{00000000-0004-0000-0500-000009000000}"/>
+    <hyperlink ref="G15" r:id="rId11" xr:uid="{00000000-0004-0000-0500-00000A000000}"/>
+    <hyperlink ref="G17" r:id="rId12" xr:uid="{00000000-0004-0000-0500-00000B000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2742,76 +3365,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="36" t="s">
-        <v>104</v>
+      <c r="A2" s="46" t="s">
+        <v>152</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="C2" s="18">
-        <v>1</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="21">
+        <v>2</v>
+      </c>
+      <c r="D2" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="24">
         <v>1350</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="24">
         <f>C2*E2</f>
-        <v>1350</v>
+        <v>2700</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>107</v>
+        <v>154</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="37" t="s">
-        <v>104</v>
+      <c r="A3" s="47" t="s">
+        <v>152</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="C3" s="18"/>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
       <c r="G3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>86</v>
+        <v>41</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2819,138 +3442,138 @@
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="48" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="C5" s="18">
         <v>6</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="D5" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="24">
         <v>497.7</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="24">
         <f>C5*E5</f>
         <v>2986.2</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="23" t="s">
-        <v>110</v>
+      <c r="G5" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="49" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>111</v>
+        <v>159</v>
       </c>
       <c r="C6" s="18">
         <v>1</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E6" s="21">
+      <c r="D6" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="E6" s="24">
         <v>299</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="24">
         <f>C6*E6</f>
         <v>299</v>
       </c>
-      <c r="G6" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>112</v>
+      <c r="G6" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="49" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="C7" s="18">
         <v>10</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="21">
+      <c r="D7" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="24">
         <v>28.35</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="24">
         <f>C7*E7</f>
         <v>283.5</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>114</v>
+      <c r="G7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="49" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="C8" s="18">
         <v>4</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="D8" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="24">
         <v>29.25</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="24">
         <f>C8*E8</f>
         <v>117</v>
       </c>
-      <c r="G8" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>116</v>
+      <c r="G8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="49" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="C9" s="18">
         <v>20</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="E9" s="21">
-        <v>0</v>
-      </c>
-      <c r="F9" s="21">
+      <c r="D9" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="24">
+        <v>29.61</v>
+      </c>
+      <c r="F9" s="24">
         <f>C9*E9</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>119</v>
+        <v>592.20000000000005</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="29" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2958,34 +3581,34 @@
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="40"/>
+      <c r="A11" s="50"/>
       <c r="B11" s="18"/>
       <c r="C11" s="18"/>
       <c r="D11" s="18"/>
-      <c r="E11" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="21"/>
+      <c r="E11" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="24"/>
       <c r="G11" s="18"/>
-      <c r="H11" s="27">
+      <c r="H11" s="37">
         <f>SUM(F2:F9)</f>
-        <v>5035.7</v>
+        <v>6977.9</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
-    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
-    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="G6" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
+    <hyperlink ref="G7" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
+    <hyperlink ref="G8" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
+    <hyperlink ref="G9" r:id="rId5" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2999,76 +3622,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1">
-      <c r="A1" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="19" t="s">
+      <c r="A1" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="36" t="s">
-        <v>104</v>
+      <c r="A2" s="46" t="s">
+        <v>152</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="C2" s="18">
-        <v>1</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="21">
+        <v>2</v>
+      </c>
+      <c r="D2" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="24">
         <v>1350</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="24">
         <f>C2*E2</f>
-        <v>1350</v>
+        <v>2700</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>107</v>
+        <v>154</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="37" t="s">
-        <v>104</v>
+      <c r="A3" s="47" t="s">
+        <v>152</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="C3" s="18"/>
-      <c r="D3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="D3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
       <c r="G3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>86</v>
+        <v>41</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3076,175 +3699,175 @@
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="51" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>120</v>
+        <v>167</v>
       </c>
       <c r="C5" s="18">
         <v>16</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="D5" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="24">
         <v>160</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="24">
         <f>C5*E5</f>
         <v>2560</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="H5" s="23" t="s">
-        <v>122</v>
+      <c r="G5" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>123</v>
+        <v>169</v>
       </c>
       <c r="C6" s="18">
         <v>3</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
+      <c r="D6" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
       <c r="G6" s="18" t="s">
-        <v>125</v>
-      </c>
-      <c r="H6" s="23" t="s">
-        <v>126</v>
+        <v>171</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>111</v>
+        <v>159</v>
       </c>
       <c r="C7" s="18">
         <v>1</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E7" s="21">
+      <c r="D7" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="24">
         <v>299</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="24">
         <f>C7*E7</f>
         <v>299</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>127</v>
+      <c r="G7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="C8" s="18">
         <v>10</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="D8" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="24">
         <v>28.35</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="24">
         <f>C8*E8</f>
         <v>283.5</v>
       </c>
-      <c r="G8" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>128</v>
+      <c r="G8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="C9" s="18">
         <v>4</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
+      <c r="D9" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
       <c r="G9" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>130</v>
+        <v>41</v>
+      </c>
+      <c r="H9" s="29" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="C10" s="18">
         <v>20</v>
       </c>
-      <c r="D10" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="E10" s="21">
-        <v>0</v>
-      </c>
-      <c r="F10" s="21">
+      <c r="D10" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="24">
+        <v>29.61</v>
+      </c>
+      <c r="F10" s="24">
         <f>C10*E10</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>127</v>
+        <v>592.20000000000005</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="29" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="C11" s="18"/>
-      <c r="D11" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
+      <c r="D11" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
       <c r="G11" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="23" t="s">
-        <v>132</v>
+        <v>41</v>
+      </c>
+      <c r="H11" s="29" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3252,26 +3875,26 @@
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="43"/>
+      <c r="A13" s="53"/>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
       <c r="D13" s="18"/>
-      <c r="E13" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="21"/>
+      <c r="E13" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="24"/>
       <c r="G13" s="18"/>
-      <c r="H13" s="27">
+      <c r="H13" s="37">
         <f>SUM(F2:F11)</f>
-        <v>4492.5</v>
+        <v>6434.7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
-    <hyperlink ref="G7" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
-    <hyperlink ref="G8" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
-    <hyperlink ref="G10" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="G7" r:id="rId2" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
+    <hyperlink ref="G8" r:id="rId3" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
+    <hyperlink ref="G10" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Omdøb hus-væg V5→V4 (global swap V4↔V5)
Partition bliver V4, yardens højre gavl bliver V5, så huset hedder rent
V1-V4 og det globale princip "ét nummer = én væg" bevares. Numrene er nu
geometrisk ordnet langs X: V3 (venstre) → V4 (partition) → V5 (højre).

Ren label-/dokumentationsændring: kun kommentarer (.scad), markdown (docs),
.py-kommentarer og 15 xlsx-celler. Ingen kode-symboler eller geometri ændret
(OpenSCAD-render verificeret identisk). 33 filer, symmetrisk 201/201 diff.
</commit_message>
<xml_diff>
--- a/docs/materialeliste.xlsx
+++ b/docs/materialeliste.xlsx
@@ -785,6 +785,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -809,6 +810,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20.1" customHeight="1" s="70">
       <c r="A6" s="75" t="inlineStr">
         <is>
@@ -871,6 +873,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="20.1" customHeight="1" s="70">
       <c r="A13" s="75" t="inlineStr">
         <is>
@@ -949,6 +952,7 @@
       </c>
       <c r="D17" s="18" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="75" t="inlineStr">
         <is>
@@ -1560,6 +1564,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="21.95" customHeight="1" s="70">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -1865,7 +1870,7 @@
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>est. — bundrem-fast: 2 på V1, 2 på V2, 3 på V3, 3 på V5</t>
+          <t>est. — bundrem-fast: 2 på V1, 2 på V2, 3 på V3, 3 på V4</t>
         </is>
       </c>
       <c r="I10" s="25" t="inlineStr">
@@ -1934,6 +1939,7 @@
       <c r="H12" s="18" t="n"/>
       <c r="I12" s="18" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14" ht="20.1" customHeight="1" s="70">
       <c r="A14" s="68" t="inlineStr">
         <is>
@@ -2066,7 +2072,7 @@
       </c>
       <c r="H17" s="24" t="inlineStr">
         <is>
-          <t>V3 + V5 bundrem</t>
+          <t>V3 + V4 bundrem</t>
         </is>
       </c>
       <c r="I17" s="25" t="inlineStr">
@@ -2150,7 +2156,7 @@
       </c>
       <c r="H19" s="24" t="inlineStr">
         <is>
-          <t>Studs V1[0..hl]+V2[0..hl]+V3+V5 + skrå toprem V3+V5 + headers/cripples</t>
+          <t>Studs V1[0..hl]+V2[0..hl]+V3+V4 + skrå toprem V3+V4 + headers/cripples</t>
         </is>
       </c>
       <c r="I19" s="25" t="inlineStr">
@@ -2177,6 +2183,7 @@
       <c r="H20" s="18" t="n"/>
       <c r="I20" s="18" t="n"/>
     </row>
+    <row r="21"/>
     <row r="22" ht="20.1" customHeight="1" s="70">
       <c r="A22" s="71" t="inlineStr">
         <is>
@@ -2529,6 +2536,7 @@
       <c r="H31" s="18" t="n"/>
       <c r="I31" s="18" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33" ht="20.1" customHeight="1" s="70">
       <c r="A33" s="65" t="inlineStr">
         <is>
@@ -2772,6 +2780,8 @@
       <c r="H39" s="18" t="n"/>
       <c r="I39" s="18" t="n"/>
     </row>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42" ht="26.1" customHeight="1" s="70">
       <c r="A42" s="18" t="n"/>
       <c r="B42" s="18" t="n"/>
@@ -2853,6 +2863,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="21.95" customHeight="1" s="70">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -2990,7 +3001,7 @@
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>3-sidet ring (V5 = hus), 4 skifter halvstensforbandt — 80 + 6 buffer</t>
+          <t>3-sidet ring (V4 = hus), 4 skifter halvstensforbandt — 80 + 6 buffer</t>
         </is>
       </c>
       <c r="I6" s="38" t="inlineStr">
@@ -3158,7 +3169,7 @@
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>est. — 4 på V1, 4 på V2, 2 på V4</t>
+          <t>est. — 4 på V1, 4 på V2, 2 på V5</t>
         </is>
       </c>
       <c r="I10" s="38" t="inlineStr">
@@ -3227,6 +3238,7 @@
       <c r="H12" s="18" t="n"/>
       <c r="I12" s="18" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14" ht="20.1" customHeight="1" s="70">
       <c r="A14" s="68" t="inlineStr">
         <is>
@@ -3359,7 +3371,7 @@
       </c>
       <c r="H17" s="24" t="inlineStr">
         <is>
-          <t>V1[2] + V2[2] + V4 bundrem</t>
+          <t>V1[2] + V2[2] + V5 bundrem</t>
         </is>
       </c>
       <c r="I17" s="38" t="inlineStr">
@@ -3485,7 +3497,7 @@
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>Studs V1[hl..ll]+V2[hl..ll]+V4 + skrå toprem V4 + yard-dør jamber</t>
+          <t>Studs V1[hl..ll]+V2[hl..ll]+V5 + skrå toprem V5 + yard-dør jamber</t>
         </is>
       </c>
       <c r="I20" s="38" t="inlineStr">
@@ -3512,6 +3524,7 @@
       <c r="H21" s="18" t="n"/>
       <c r="I21" s="18" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="20.1" customHeight="1" s="70">
       <c r="A23" s="71" t="inlineStr">
         <is>
@@ -3864,6 +3877,7 @@
       <c r="H32" s="18" t="n"/>
       <c r="I32" s="18" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34" ht="20.1" customHeight="1" s="70">
       <c r="A34" s="65" t="inlineStr">
         <is>
@@ -3974,6 +3988,8 @@
       <c r="H37" s="18" t="n"/>
       <c r="I37" s="18" t="n"/>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40" ht="26.1" customHeight="1" s="70">
       <c r="A40" s="18" t="n"/>
       <c r="B40" s="18" t="n"/>
@@ -4054,6 +4070,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="20.1" customHeight="1" s="70">
       <c r="A3" s="39" t="inlineStr">
         <is>
@@ -4426,6 +4443,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="75" t="inlineStr">
         <is>
@@ -4715,7 +4734,7 @@
       </c>
       <c r="H5" s="24" t="inlineStr">
         <is>
-          <t>3-sidet ring (V5 = hus), 4 skifter halvstensforbandt — 80 + 6 buffer</t>
+          <t>3-sidet ring (V4 = hus), 4 skifter halvstensforbandt — 80 + 6 buffer</t>
         </is>
       </c>
       <c r="I5" s="38" t="inlineStr">
@@ -5009,7 +5028,7 @@
       </c>
       <c r="H12" s="24" t="inlineStr">
         <is>
-          <t>est. — bundrem-fast: 2 på V1, 2 på V2, 3 på V3, 3 på V5</t>
+          <t>est. — bundrem-fast: 2 på V1, 2 på V2, 3 på V3, 3 på V4</t>
         </is>
       </c>
       <c r="I12" s="25" t="inlineStr">
@@ -5051,7 +5070,7 @@
       </c>
       <c r="H13" s="24" t="inlineStr">
         <is>
-          <t>est. — 4 på V1, 4 på V2, 2 på V4</t>
+          <t>est. — 4 på V1, 4 på V2, 2 på V5</t>
         </is>
       </c>
       <c r="I13" s="38" t="inlineStr">
@@ -5423,7 +5442,7 @@
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
-          <t>V3 + V5 bundrem</t>
+          <t>V3 + V4 bundrem</t>
         </is>
       </c>
       <c r="I4" s="25" t="inlineStr">
@@ -5465,7 +5484,7 @@
       </c>
       <c r="H5" s="24" t="inlineStr">
         <is>
-          <t>V1[2] + V2[2] + V4 bundrem</t>
+          <t>V1[2] + V2[2] + V5 bundrem</t>
         </is>
       </c>
       <c r="I5" s="38" t="inlineStr">
@@ -5591,7 +5610,7 @@
       </c>
       <c r="H8" s="24" t="inlineStr">
         <is>
-          <t>Studs V1[0..hl]+V2[0..hl]+V3+V5 + skrå toprem V3+V5 + headers/cripples</t>
+          <t>Studs V1[0..hl]+V2[0..hl]+V3+V4 + skrå toprem V3+V4 + headers/cripples</t>
         </is>
       </c>
       <c r="I8" s="25" t="inlineStr">
@@ -5633,7 +5652,7 @@
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
-          <t>Studs V1[hl..ll]+V2[hl..ll]+V4 + skrå toprem V4 + yard-dør jamber</t>
+          <t>Studs V1[hl..ll]+V2[hl..ll]+V5 + skrå toprem V5 + yard-dør jamber</t>
         </is>
       </c>
       <c r="I9" s="38" t="inlineStr">
@@ -5874,7 +5893,7 @@
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
-          <t>X=1800..5400 + V4 gable + vindskede H</t>
+          <t>X=1800..5400 + V5 gable + vindskede H</t>
         </is>
       </c>
       <c r="I3" s="38" t="inlineStr">

</xml_diff>